<commit_message>
feat(api): enhance workbook upload with preview option and add attachment handling
- Updated `uploadWorkbook` function to include a `preview` parameter for conditional endpoint selection.
- Added `downloadWorkbook` function for exporting workbooks.
- Introduced `uploadAttachment` function for attaching files to specific records.
- Implemented `downloadAttachment` function for retrieving attachments.

style(css): improve UI styles for better usability and responsiveness

- Added new styles for preview sheets, record previews, and attachment management.
- Enhanced button styles and layout for better user interaction.
- Improved responsiveness for various components on smaller screens.
</commit_message>
<xml_diff>
--- a/Business.xlsx
+++ b/Business.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,16 +28,26 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="0017211c"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ffffff"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +55,14 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -416,28 +428,36 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col hidden="1" width="13" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>__ledgerly_record_id</t>
         </is>
       </c>
     </row>
@@ -452,33 +472,41 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col hidden="1" width="13" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Bill</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Paid</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Balance</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>__ledgerly_record_id</t>
         </is>
       </c>
     </row>
@@ -493,8 +521,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col hidden="1" width="13" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -515,6 +546,11 @@
       <c r="D1" t="inlineStr">
         <is>
           <t>Email</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>__ledgerly_record_id</t>
         </is>
       </c>
     </row>
@@ -529,28 +565,37 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col hidden="1" width="13" customWidth="1" min="5" max="5"/>
+    <col hidden="1" width="13" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Due Date</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>__ledgerly_record_id</t>
         </is>
       </c>
     </row>

</xml_diff>